<commit_message>
added 2k-5k comparison lab
</commit_message>
<xml_diff>
--- a/SAC_result_multiW_5k.xlsx
+++ b/SAC_result_multiW_5k.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Semester\SemesterVII\thesis_1228\lab\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C7D5612-C482-4678-A1AE-44DAF06A30BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F93A771-B7C7-44B0-97CB-367EFBF0E416}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="203">
   <si>
     <t>Queen</t>
   </si>
@@ -364,31 +364,40 @@
     <t>lambda</t>
   </si>
   <si>
-    <t>0.070</t>
-  </si>
-  <si>
-    <t>0.038</t>
-  </si>
-  <si>
-    <t>-0.009</t>
-  </si>
-  <si>
-    <t>0.104</t>
-  </si>
-  <si>
-    <t>0.190</t>
-  </si>
-  <si>
-    <t>0.323</t>
-  </si>
-  <si>
-    <t>0.339</t>
-  </si>
-  <si>
-    <t>0.389</t>
-  </si>
-  <si>
-    <t>0.388</t>
+    <t>0.070**
+(0.032)</t>
+  </si>
+  <si>
+    <t>0.038***
+(0.004)</t>
+  </si>
+  <si>
+    <t>-0.009
+(0.024)</t>
+  </si>
+  <si>
+    <t>0.104***
+(0.031)</t>
+  </si>
+  <si>
+    <t>0.190***
+(0.035)</t>
+  </si>
+  <si>
+    <t>0.323***
+(0.038)</t>
+  </si>
+  <si>
+    <t>0.339***
+(0.037)</t>
+  </si>
+  <si>
+    <t>0.389***
+(0.042)</t>
+  </si>
+  <si>
+    <t>0.388***
+(0.044)</t>
   </si>
   <si>
     <t>Residual Moran's I</t>
@@ -463,91 +472,91 @@
     <t>Log Likelihood</t>
   </si>
   <si>
-    <t>-228.813</t>
-  </si>
-  <si>
-    <t>-242.422</t>
-  </si>
-  <si>
-    <t>-236.751</t>
-  </si>
-  <si>
-    <t>-238.905</t>
-  </si>
-  <si>
-    <t>-239.211</t>
-  </si>
-  <si>
-    <t>-242.253</t>
-  </si>
-  <si>
-    <t>-241.487</t>
-  </si>
-  <si>
-    <t>-243.697</t>
-  </si>
-  <si>
-    <t>-245.797</t>
+    <t>-233.996</t>
+  </si>
+  <si>
+    <t>-242.532</t>
+  </si>
+  <si>
+    <t>-238.753</t>
+  </si>
+  <si>
+    <t>-239.984</t>
+  </si>
+  <si>
+    <t>-240.519</t>
+  </si>
+  <si>
+    <t>-244.072</t>
+  </si>
+  <si>
+    <t>-243.303</t>
+  </si>
+  <si>
+    <t>-245.626</t>
+  </si>
+  <si>
+    <t>-247.556</t>
   </si>
   <si>
     <t>Akaike Info Criterion</t>
   </si>
   <si>
-    <t>473.625</t>
-  </si>
-  <si>
-    <t>500.844</t>
-  </si>
-  <si>
-    <t>489.502</t>
-  </si>
-  <si>
-    <t>493.810</t>
-  </si>
-  <si>
-    <t>494.422</t>
-  </si>
-  <si>
-    <t>500.505</t>
-  </si>
-  <si>
-    <t>498.973</t>
-  </si>
-  <si>
-    <t>503.394</t>
-  </si>
-  <si>
-    <t>507.594</t>
+    <t>483.991</t>
+  </si>
+  <si>
+    <t>501.064</t>
+  </si>
+  <si>
+    <t>493.505</t>
+  </si>
+  <si>
+    <t>495.968</t>
+  </si>
+  <si>
+    <t>497.039</t>
+  </si>
+  <si>
+    <t>504.144</t>
+  </si>
+  <si>
+    <t>502.606</t>
+  </si>
+  <si>
+    <t>507.253</t>
+  </si>
+  <si>
+    <t>511.112</t>
   </si>
   <si>
     <t>Schwarz Criterion</t>
   </si>
   <si>
-    <t>499.931</t>
-  </si>
-  <si>
-    <t>527.151</t>
-  </si>
-  <si>
-    <t>515.808</t>
-  </si>
-  <si>
-    <t>520.116</t>
-  </si>
-  <si>
-    <t>520.728</t>
-  </si>
-  <si>
-    <t>526.811</t>
-  </si>
-  <si>
-    <t>525.279</t>
-  </si>
-  <si>
-    <t>529.700</t>
-  </si>
-  <si>
-    <t>533.900</t>
+    <t>510.298</t>
+  </si>
+  <si>
+    <t>527.370</t>
+  </si>
+  <si>
+    <t>519.811</t>
+  </si>
+  <si>
+    <t>522.274</t>
+  </si>
+  <si>
+    <t>523.345</t>
+  </si>
+  <si>
+    <t>530.450</t>
+  </si>
+  <si>
+    <t>528.912</t>
+  </si>
+  <si>
+    <t>533.559</t>
+  </si>
+  <si>
+    <t>537.418</t>
   </si>
   <si>
     <t>Wald</t>
@@ -607,85 +616,76 @@
     <t>LR_SAR</t>
   </si>
   <si>
-    <t>9.632</t>
-  </si>
-  <si>
-    <t>0.067</t>
-  </si>
-  <si>
-    <t>3.882</t>
-  </si>
-  <si>
-    <t>1.160</t>
-  </si>
-  <si>
-    <t>-0.164</t>
-  </si>
-  <si>
-    <t>-6.109</t>
-  </si>
-  <si>
-    <t>-4.764</t>
-  </si>
-  <si>
-    <t>-6.366</t>
-  </si>
-  <si>
-    <t>-6.993</t>
+    <t>-0.734</t>
+  </si>
+  <si>
+    <t>-0.153</t>
+  </si>
+  <si>
+    <t>-0.121</t>
+  </si>
+  <si>
+    <t>-0.998</t>
+  </si>
+  <si>
+    <t>-2.781</t>
+  </si>
+  <si>
+    <t>-9.748</t>
+  </si>
+  <si>
+    <t>-8.397</t>
+  </si>
+  <si>
+    <t>-10.225</t>
+  </si>
+  <si>
+    <t>-10.512</t>
   </si>
   <si>
     <t>LR_SAR_p</t>
   </si>
   <si>
-    <t>0.141</t>
-  </si>
-  <si>
-    <t>0.693</t>
-  </si>
-  <si>
     <t>LR_SEM</t>
   </si>
   <si>
-    <t>12.483</t>
-  </si>
-  <si>
-    <t>1.280</t>
-  </si>
-  <si>
-    <t>5.916</t>
-  </si>
-  <si>
-    <t>1.049</t>
-  </si>
-  <si>
-    <t>-1.435</t>
-  </si>
-  <si>
-    <t>-9.856</t>
-  </si>
-  <si>
-    <t>-8.797</t>
-  </si>
-  <si>
-    <t>-11.282</t>
-  </si>
-  <si>
-    <t>-11.441</t>
+    <t>2.116</t>
+  </si>
+  <si>
+    <t>1.060</t>
+  </si>
+  <si>
+    <t>1.913</t>
+  </si>
+  <si>
+    <t>-1.108</t>
+  </si>
+  <si>
+    <t>-4.052</t>
+  </si>
+  <si>
+    <t>-13.495</t>
+  </si>
+  <si>
+    <t>-12.430</t>
+  </si>
+  <si>
+    <t>-15.141</t>
+  </si>
+  <si>
+    <t>-14.959</t>
   </si>
   <si>
     <t>LR_SEM_p</t>
   </si>
   <si>
-    <t>0.052</t>
-  </si>
-  <si>
-    <t>0.973</t>
-  </si>
-  <si>
-    <t>0.433</t>
-  </si>
-  <si>
-    <t>0.984</t>
+    <t>0.909</t>
+  </si>
+  <si>
+    <t>0.983</t>
+  </si>
+  <si>
+    <t>0.928</t>
   </si>
   <si>
     <t>Lagrange Multiplier (LM)</t>
@@ -1383,7 +1383,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="10" spans="1:10">
+    <row r="10" spans="1:10" ht="28">
       <c r="A10" s="1" t="s">
         <v>89</v>
       </c>
@@ -1676,16 +1676,16 @@
         <v>177</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>178</v>
+        <v>165</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>165</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>179</v>
+        <v>165</v>
       </c>
       <c r="E19" s="2" t="s">
-        <v>161</v>
+        <v>165</v>
       </c>
       <c r="F19" s="2" t="s">
         <v>165</v>
@@ -1705,51 +1705,51 @@
     </row>
     <row r="20" spans="1:10">
       <c r="A20" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>179</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="E20" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="D20" s="2" t="s">
+      <c r="F20" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="G20" s="2" t="s">
         <v>184</v>
       </c>
-      <c r="F20" s="2" t="s">
+      <c r="H20" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="G20" s="2" t="s">
+      <c r="I20" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="H20" s="2" t="s">
+      <c r="J20" s="2" t="s">
         <v>187</v>
-      </c>
-      <c r="I20" s="2" t="s">
-        <v>188</v>
-      </c>
-      <c r="J20" s="2" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="21" spans="1:10">
       <c r="A21" s="1" t="s">
+        <v>188</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>189</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="D21" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>192</v>
-      </c>
-      <c r="D21" s="2" t="s">
-        <v>193</v>
-      </c>
       <c r="E21" s="2" t="s">
-        <v>194</v>
+        <v>165</v>
       </c>
       <c r="F21" s="2" t="s">
         <v>165</v>
@@ -1769,39 +1769,39 @@
     </row>
     <row r="22" spans="1:10" ht="42">
       <c r="A22" s="1" t="s">
+        <v>192</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>193</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>194</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="E22" s="2" t="s">
         <v>196</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="F22" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="D22" s="2" t="s">
+      <c r="G22" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="H22" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="F22" s="2" t="s">
+      <c r="I22" s="2" t="s">
         <v>200</v>
       </c>
-      <c r="G22" s="2" t="s">
+      <c r="J22" s="2" t="s">
         <v>201</v>
-      </c>
-      <c r="H22" s="2" t="s">
-        <v>202</v>
-      </c>
-      <c r="I22" s="2" t="s">
-        <v>203</v>
-      </c>
-      <c r="J22" s="2" t="s">
-        <v>204</v>
       </c>
     </row>
     <row r="23" spans="1:10" ht="28">
       <c r="A23" s="1" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>80</v>

</xml_diff>